<commit_message>
new images css most comprised
</commit_message>
<xml_diff>
--- a/Bufanda Bilduma.xlsx
+++ b/Bufanda Bilduma.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andmu\Documents\Andoni\kodea\bufandaweb\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Kodea\Beste\bufandaweb2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5338BCEE-77DF-4930-BA9A-02A16CB9000D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="584">
   <si>
     <t>ZENBAKIA</t>
   </si>
@@ -1753,9 +1752,6 @@
     <t>arconada_cruiff.jpg</t>
   </si>
   <si>
-    <t>arconda_cruiff_arconada.jpg</t>
-  </si>
-  <si>
     <t>cracovia_eskudo.jpg</t>
   </si>
   <si>
@@ -1781,13 +1777,76 @@
   </si>
   <si>
     <t>David eta Iñakiren opari bat. Oso gutxi egin zituzten eta Ajaxeko zeleek etengabe eskatu zizkieten.</t>
+  </si>
+  <si>
+    <t>arconada_cruiff_arconada.jpg</t>
+  </si>
+  <si>
+    <t>Miguel Galarraga</t>
+  </si>
+  <si>
+    <t>Nereak Bostonen egindako ikerketa estantziatik ekarria</t>
+  </si>
+  <si>
+    <t>new_england_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>new_england.jpg</t>
+  </si>
+  <si>
+    <t>new_england_atze.jpg</t>
+  </si>
+  <si>
+    <t>Errumania</t>
+  </si>
+  <si>
+    <t>2025 Ekaina</t>
+  </si>
+  <si>
+    <t>Cluj</t>
+  </si>
+  <si>
+    <t>Sibiu</t>
+  </si>
+  <si>
+    <t>Itziarrek kongresu batetik ekarritakoa</t>
+  </si>
+  <si>
+    <t>lokomotive_leipzig_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>lokomotive_leipzig.jpeg</t>
+  </si>
+  <si>
+    <t>hermanstadt_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>hermanstadt.jpg</t>
+  </si>
+  <si>
+    <t>hermanstadt_atze.jpg</t>
+  </si>
+  <si>
+    <t>cluj_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>cluj.jpg</t>
+  </si>
+  <si>
+    <t>cluj_atze.jpg</t>
+  </si>
+  <si>
+    <t>atlanta_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>atlanta.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="9" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2398,7 +2457,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle name="Sheet1-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="Sheet1-style" pivot="0" count="3">
       <tableStyleElement type="headerRow" dxfId="3"/>
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="secondRowStripe" dxfId="1"/>
@@ -2416,19 +2475,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K213">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:K213">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ZENBAKIA" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="TALDEA"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="NONDIK"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="LIGA"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="NORK"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="NOIZ"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="BESTE"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="main_image"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="image_1"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="image_2"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="image_3"/>
+    <tableColumn id="1" name="ZENBAKIA" dataDxfId="0"/>
+    <tableColumn id="2" name="TALDEA"/>
+    <tableColumn id="3" name="NONDIK"/>
+    <tableColumn id="4" name="LIGA"/>
+    <tableColumn id="5" name="NORK"/>
+    <tableColumn id="6" name="NOIZ"/>
+    <tableColumn id="7" name="BESTE"/>
+    <tableColumn id="8" name="main_image"/>
+    <tableColumn id="9" name="image_1"/>
+    <tableColumn id="10" name="image_2"/>
+    <tableColumn id="11" name="image_3"/>
   </tableColumns>
   <tableStyleInfo name="Sheet1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2750,12 +2809,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K215"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:K217"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="16" customWidth="1"/>
     <col min="2" max="2" width="40.28515625" bestFit="1" customWidth="1"/>
@@ -2770,7 +2829,7 @@
     <col min="11" max="11" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -2805,7 +2864,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -2825,7 +2884,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1">
       <c r="A3" s="12">
         <v>2</v>
       </c>
@@ -2845,7 +2904,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1">
       <c r="A4" s="12">
         <v>3</v>
       </c>
@@ -2865,7 +2924,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -2885,7 +2944,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="15.75" customHeight="1">
       <c r="A6" s="12">
         <v>5</v>
       </c>
@@ -2905,7 +2964,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -2922,7 +2981,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="15.75" customHeight="1">
       <c r="A8" s="12">
         <v>7</v>
       </c>
@@ -2939,7 +2998,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="15.75" customHeight="1">
       <c r="A9" s="12">
         <v>8</v>
       </c>
@@ -2959,7 +3018,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="15.75" customHeight="1">
       <c r="A10" s="12">
         <v>9</v>
       </c>
@@ -2979,7 +3038,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="15.75" customHeight="1">
       <c r="A11" s="12">
         <v>10</v>
       </c>
@@ -2999,7 +3058,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="15.75" customHeight="1">
       <c r="A12" s="12">
         <v>11</v>
       </c>
@@ -3016,7 +3075,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="15.75" customHeight="1">
       <c r="A13" s="12">
         <v>12</v>
       </c>
@@ -3033,7 +3092,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="15.75" customHeight="1">
       <c r="A14" s="12">
         <v>13</v>
       </c>
@@ -3053,7 +3112,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" ht="15.75" customHeight="1">
       <c r="A15" s="12">
         <v>14</v>
       </c>
@@ -3073,7 +3132,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" ht="15.75" customHeight="1">
       <c r="A16" s="12">
         <v>15</v>
       </c>
@@ -3093,7 +3152,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1">
       <c r="A17" s="12">
         <v>16</v>
       </c>
@@ -3107,7 +3166,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1">
       <c r="A18" s="12">
         <v>17</v>
       </c>
@@ -3127,7 +3186,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="15.75" customHeight="1">
       <c r="A19" s="12">
         <v>18</v>
       </c>
@@ -3144,7 +3203,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1">
       <c r="A20" s="12">
         <v>19</v>
       </c>
@@ -3161,7 +3220,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1">
       <c r="A21" s="12">
         <v>20</v>
       </c>
@@ -3181,7 +3240,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1">
       <c r="A22" s="12">
         <v>21</v>
       </c>
@@ -3201,7 +3260,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1">
       <c r="A23" s="12">
         <v>22</v>
       </c>
@@ -3221,7 +3280,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1">
       <c r="A24" s="12">
         <v>23</v>
       </c>
@@ -3238,7 +3297,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1">
       <c r="A25" s="12">
         <v>24</v>
       </c>
@@ -3255,7 +3314,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="15.75" customHeight="1">
       <c r="A26" s="12">
         <v>25</v>
       </c>
@@ -3275,7 +3334,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1">
       <c r="A27" s="12">
         <v>26</v>
       </c>
@@ -3295,7 +3354,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1">
       <c r="A28" s="12">
         <v>27</v>
       </c>
@@ -3312,7 +3371,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1">
       <c r="A29" s="12">
         <v>28</v>
       </c>
@@ -3329,7 +3388,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1">
       <c r="A30" s="12">
         <v>29</v>
       </c>
@@ -3346,7 +3405,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" ht="15.75" customHeight="1">
       <c r="A31" s="12">
         <v>30</v>
       </c>
@@ -3363,7 +3422,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" ht="15.75" customHeight="1">
       <c r="A32" s="12">
         <v>31</v>
       </c>
@@ -3380,7 +3439,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="15.75" customHeight="1">
       <c r="A33" s="12">
         <v>32</v>
       </c>
@@ -3400,7 +3459,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="15.75" customHeight="1">
       <c r="A34" s="12">
         <v>33</v>
       </c>
@@ -3420,7 +3479,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="15.75" customHeight="1">
       <c r="A35" s="12">
         <v>34</v>
       </c>
@@ -3437,7 +3496,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="15.75" customHeight="1">
       <c r="A36" s="12">
         <v>35</v>
       </c>
@@ -3457,7 +3516,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" ht="15.75" customHeight="1">
       <c r="A37" s="12">
         <v>36</v>
       </c>
@@ -3477,7 +3536,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" ht="12.75">
       <c r="A38" s="12">
         <v>37</v>
       </c>
@@ -3497,7 +3556,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ht="12.75">
       <c r="A39" s="12">
         <v>38</v>
       </c>
@@ -3514,7 +3573,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" ht="12.75">
       <c r="A40" s="12">
         <v>39</v>
       </c>
@@ -3534,7 +3593,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" ht="12.75">
       <c r="A41" s="12">
         <v>40</v>
       </c>
@@ -3554,7 +3613,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" ht="12.75">
       <c r="A42" s="12">
         <v>41</v>
       </c>
@@ -3571,7 +3630,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" ht="12.75">
       <c r="A43" s="12">
         <v>42</v>
       </c>
@@ -3591,7 +3650,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" ht="12.75">
       <c r="A44" s="12">
         <v>43</v>
       </c>
@@ -3611,7 +3670,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" ht="12.75">
       <c r="A45" s="12">
         <v>44</v>
       </c>
@@ -3631,7 +3690,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" ht="12.75">
       <c r="A46" s="12">
         <v>45</v>
       </c>
@@ -3648,7 +3707,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" ht="12.75">
       <c r="A47" s="12">
         <v>46</v>
       </c>
@@ -3665,7 +3724,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" ht="12.75">
       <c r="A48" s="12">
         <v>47</v>
       </c>
@@ -3685,7 +3744,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" ht="12.75">
       <c r="A49" s="12">
         <v>48</v>
       </c>
@@ -3702,7 +3761,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" ht="12.75">
       <c r="A50" s="12">
         <v>49</v>
       </c>
@@ -3722,7 +3781,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" ht="12.75">
       <c r="A51" s="12">
         <v>50</v>
       </c>
@@ -3742,7 +3801,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" ht="12.75">
       <c r="A52" s="12">
         <v>51</v>
       </c>
@@ -3759,7 +3818,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" ht="12.75">
       <c r="A53" s="12">
         <v>52</v>
       </c>
@@ -3779,7 +3838,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" ht="12.75">
       <c r="A54" s="12">
         <v>53</v>
       </c>
@@ -3796,7 +3855,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" ht="12.75">
       <c r="A55" s="12">
         <v>54</v>
       </c>
@@ -3816,7 +3875,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" ht="12.75">
       <c r="A56" s="12">
         <v>55</v>
       </c>
@@ -3836,7 +3895,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" ht="12.75">
       <c r="A57" s="12">
         <v>56</v>
       </c>
@@ -3856,7 +3915,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" ht="12.75">
       <c r="A58" s="12">
         <v>57</v>
       </c>
@@ -3876,7 +3935,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" ht="12.75">
       <c r="A59" s="12">
         <v>58</v>
       </c>
@@ -3893,7 +3952,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" ht="12.75">
       <c r="A60" s="12">
         <v>59</v>
       </c>
@@ -3910,7 +3969,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" ht="12.75">
       <c r="A61" s="12">
         <v>60</v>
       </c>
@@ -3930,7 +3989,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" ht="12.75">
       <c r="A62" s="12">
         <v>61</v>
       </c>
@@ -3950,7 +4009,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" ht="12.75">
       <c r="A63" s="12">
         <v>62</v>
       </c>
@@ -3970,7 +4029,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" ht="12.75">
       <c r="A64" s="12">
         <v>63</v>
       </c>
@@ -3990,7 +4049,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" ht="12.75">
       <c r="A65" s="12">
         <v>64</v>
       </c>
@@ -4010,7 +4069,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" ht="12.75">
       <c r="A66" s="12">
         <v>65</v>
       </c>
@@ -4030,7 +4089,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" ht="12.75">
       <c r="A67" s="12">
         <v>66</v>
       </c>
@@ -4050,7 +4109,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" ht="12.75">
       <c r="A68" s="12">
         <v>67</v>
       </c>
@@ -4070,7 +4129,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" ht="12.75">
       <c r="A69" s="12">
         <v>68</v>
       </c>
@@ -4090,7 +4149,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" ht="12.75">
       <c r="A70" s="12">
         <v>69</v>
       </c>
@@ -4110,7 +4169,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" ht="12.75">
       <c r="A71" s="12">
         <v>70</v>
       </c>
@@ -4130,7 +4189,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" ht="12.75">
       <c r="A72" s="12">
         <v>71</v>
       </c>
@@ -4150,7 +4209,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" ht="12.75">
       <c r="A73" s="12">
         <v>72</v>
       </c>
@@ -4170,7 +4229,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" ht="12.75">
       <c r="A74" s="12">
         <v>73</v>
       </c>
@@ -4190,7 +4249,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" ht="12.75">
       <c r="A75" s="12">
         <v>74</v>
       </c>
@@ -4210,7 +4269,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" ht="12.75">
       <c r="A76" s="12">
         <v>75</v>
       </c>
@@ -4230,7 +4289,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" ht="12.75">
       <c r="A77" s="12">
         <v>76</v>
       </c>
@@ -4250,7 +4309,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" ht="12.75">
       <c r="A78" s="12">
         <v>77</v>
       </c>
@@ -4270,7 +4329,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" ht="12.75">
       <c r="A79" s="12">
         <v>78</v>
       </c>
@@ -4290,7 +4349,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" ht="12.75">
       <c r="A80" s="12">
         <v>79</v>
       </c>
@@ -4310,7 +4369,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" ht="12.75">
       <c r="A81" s="12">
         <v>80</v>
       </c>
@@ -4330,7 +4389,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" ht="12.75">
       <c r="A82" s="12">
         <v>81</v>
       </c>
@@ -4350,7 +4409,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" ht="12.75">
       <c r="A83" s="12">
         <v>82</v>
       </c>
@@ -4370,7 +4429,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" ht="12.75">
       <c r="A84" s="12">
         <v>83</v>
       </c>
@@ -4390,7 +4449,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" ht="12.75">
       <c r="A85" s="12">
         <v>84</v>
       </c>
@@ -4410,7 +4469,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" ht="12.75">
       <c r="A86" s="12">
         <v>85</v>
       </c>
@@ -4430,7 +4489,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" ht="12.75">
       <c r="A87" s="12">
         <v>86</v>
       </c>
@@ -4450,7 +4509,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" ht="12.75">
       <c r="A88" s="12">
         <v>87</v>
       </c>
@@ -4470,7 +4529,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" ht="12.75">
       <c r="A89" s="12">
         <v>88</v>
       </c>
@@ -4490,7 +4549,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" ht="12.75">
       <c r="A90" s="12">
         <v>89</v>
       </c>
@@ -4510,7 +4569,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" ht="12.75">
       <c r="A91" s="12">
         <v>90</v>
       </c>
@@ -4530,7 +4589,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" ht="12.75">
       <c r="A92" s="12">
         <v>91</v>
       </c>
@@ -4550,7 +4609,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" ht="12.75">
       <c r="A93" s="12">
         <v>92</v>
       </c>
@@ -4570,7 +4629,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" ht="12.75">
       <c r="A94" s="12">
         <v>93</v>
       </c>
@@ -4590,7 +4649,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" ht="12.75">
       <c r="A95" s="12">
         <v>94</v>
       </c>
@@ -4610,7 +4669,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" ht="12.75">
       <c r="A96" s="12">
         <v>95</v>
       </c>
@@ -4630,7 +4689,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" ht="12.75">
       <c r="A97" s="12">
         <v>96</v>
       </c>
@@ -4650,7 +4709,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" ht="12.75">
       <c r="A98" s="12">
         <v>97</v>
       </c>
@@ -4670,7 +4729,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" ht="12.75">
       <c r="A99" s="12">
         <v>98</v>
       </c>
@@ -4690,7 +4749,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" ht="12.75">
       <c r="A100" s="12">
         <v>99</v>
       </c>
@@ -4710,7 +4769,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" ht="12.75">
       <c r="A101" s="12">
         <v>100</v>
       </c>
@@ -4730,7 +4789,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" ht="12.75">
       <c r="A102" s="12">
         <v>101</v>
       </c>
@@ -4750,7 +4809,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" ht="12.75">
       <c r="A103" s="12">
         <v>102</v>
       </c>
@@ -4770,7 +4829,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" ht="12.75">
       <c r="A104" s="12">
         <v>103</v>
       </c>
@@ -4790,7 +4849,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" ht="12.75">
       <c r="A105" s="12">
         <v>104</v>
       </c>
@@ -4810,7 +4869,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" ht="12.75">
       <c r="A106" s="12">
         <v>105</v>
       </c>
@@ -4830,7 +4889,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" ht="12.75">
       <c r="A107" s="12">
         <v>106</v>
       </c>
@@ -4850,7 +4909,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" ht="12.75">
       <c r="A108" s="12">
         <v>107</v>
       </c>
@@ -4870,7 +4929,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" ht="12.75">
       <c r="A109" s="12">
         <v>108</v>
       </c>
@@ -4890,7 +4949,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" ht="12.75">
       <c r="A110" s="12">
         <v>109</v>
       </c>
@@ -4910,7 +4969,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" ht="12.75">
       <c r="A111" s="12">
         <v>110</v>
       </c>
@@ -4930,7 +4989,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" ht="12.75">
       <c r="A112" s="12">
         <v>111</v>
       </c>
@@ -4950,7 +5009,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" ht="12.75">
       <c r="A113" s="12">
         <v>112</v>
       </c>
@@ -4970,7 +5029,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="114" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" ht="12.75">
       <c r="A114" s="12">
         <v>113</v>
       </c>
@@ -4990,7 +5049,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="115" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" ht="12.75">
       <c r="A115" s="12">
         <v>114</v>
       </c>
@@ -5010,7 +5069,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" ht="12.75">
       <c r="A116" s="12">
         <v>115</v>
       </c>
@@ -5030,7 +5089,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="117" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" ht="12.75">
       <c r="A117" s="12">
         <v>116</v>
       </c>
@@ -5050,7 +5109,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" ht="12.75">
       <c r="A118" s="12">
         <v>117</v>
       </c>
@@ -5070,7 +5129,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" ht="12.75">
       <c r="A119" s="12">
         <v>118</v>
       </c>
@@ -5090,7 +5149,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" ht="12.75">
       <c r="A120" s="12">
         <v>119</v>
       </c>
@@ -5110,7 +5169,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" ht="12.75">
       <c r="A121" s="12">
         <v>120</v>
       </c>
@@ -5130,7 +5189,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" ht="12.75">
       <c r="A122" s="12">
         <v>121</v>
       </c>
@@ -5150,7 +5209,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="123" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" ht="12.75">
       <c r="A123" s="12">
         <v>122</v>
       </c>
@@ -5170,7 +5229,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="124" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" ht="12.75">
       <c r="A124" s="12">
         <v>123</v>
       </c>
@@ -5190,7 +5249,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="125" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" ht="12.75">
       <c r="A125" s="12">
         <v>124</v>
       </c>
@@ -5210,7 +5269,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="126" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" ht="12.75">
       <c r="A126" s="12">
         <v>125</v>
       </c>
@@ -5230,7 +5289,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="127" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" ht="12.75">
       <c r="A127" s="12">
         <v>126</v>
       </c>
@@ -5250,7 +5309,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="128" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" ht="12.75">
       <c r="A128" s="12">
         <v>127</v>
       </c>
@@ -5270,7 +5329,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:7" ht="12.75">
       <c r="A129" s="12">
         <v>128</v>
       </c>
@@ -5290,7 +5349,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:7" ht="12.75">
       <c r="A130" s="12">
         <v>129</v>
       </c>
@@ -5310,7 +5369,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:7" ht="12.75">
       <c r="A131" s="12">
         <v>130</v>
       </c>
@@ -5330,7 +5389,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:7" ht="12.75">
       <c r="A132" s="12">
         <v>131</v>
       </c>
@@ -5350,7 +5409,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:7" ht="12.75">
       <c r="A133" s="12">
         <v>132</v>
       </c>
@@ -5370,7 +5429,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:7" ht="12.75">
       <c r="A134" s="12">
         <v>133</v>
       </c>
@@ -5393,7 +5452,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:7" ht="12.75">
       <c r="A135" s="12">
         <v>134</v>
       </c>
@@ -5413,7 +5472,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:7" ht="12.75">
       <c r="A136" s="12">
         <v>135</v>
       </c>
@@ -5433,7 +5492,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:7" ht="12.75">
       <c r="A137" s="12">
         <v>136</v>
       </c>
@@ -5453,7 +5512,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:7" ht="12.75">
       <c r="A138" s="12">
         <v>137</v>
       </c>
@@ -5473,7 +5532,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:7" ht="12.75">
       <c r="A139" s="12">
         <v>138</v>
       </c>
@@ -5493,7 +5552,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:7" ht="12.75">
       <c r="A140" s="12">
         <v>139</v>
       </c>
@@ -5513,7 +5572,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:7" ht="12.75">
       <c r="A141" s="12">
         <v>140</v>
       </c>
@@ -5533,7 +5592,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:7" ht="12.75">
       <c r="A142" s="12">
         <v>141</v>
       </c>
@@ -5553,7 +5612,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:7" ht="12.75">
       <c r="A143" s="12">
         <v>142</v>
       </c>
@@ -5573,7 +5632,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:7" ht="12.75">
       <c r="A144" s="12">
         <v>143</v>
       </c>
@@ -5593,7 +5652,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:10" ht="12.75">
       <c r="A145" s="12">
         <v>144</v>
       </c>
@@ -5613,7 +5672,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:10" ht="12.75">
       <c r="A146" s="12">
         <v>145</v>
       </c>
@@ -5633,7 +5692,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:10" ht="12.75">
       <c r="A147" s="12">
         <v>146</v>
       </c>
@@ -5653,7 +5712,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:10" ht="12.75">
       <c r="A148" s="12">
         <v>147</v>
       </c>
@@ -5673,7 +5732,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:10" ht="12.75">
       <c r="A149" s="12">
         <v>148</v>
       </c>
@@ -5693,7 +5752,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:10" ht="12.75">
       <c r="A150" s="12">
         <v>149</v>
       </c>
@@ -5713,7 +5772,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:10" ht="12.75">
       <c r="A151" s="12">
         <v>150</v>
       </c>
@@ -5733,7 +5792,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:10" ht="12.75">
       <c r="A152" s="12">
         <v>151</v>
       </c>
@@ -5753,7 +5812,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:10" ht="12.75">
       <c r="A153" s="12">
         <v>152</v>
       </c>
@@ -5773,7 +5832,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:10" ht="12.75">
       <c r="A154" s="12">
         <v>153</v>
       </c>
@@ -5793,7 +5852,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:10" ht="12.75">
       <c r="A155" s="12">
         <v>154</v>
       </c>
@@ -5813,7 +5872,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:10" ht="12.75">
       <c r="A156" s="12">
         <v>155</v>
       </c>
@@ -5832,8 +5891,17 @@
       <c r="F156" s="3" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="157" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="G156" t="s">
+        <v>573</v>
+      </c>
+      <c r="H156" t="s">
+        <v>574</v>
+      </c>
+      <c r="I156" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" ht="12.75">
       <c r="A157" s="12">
         <v>156</v>
       </c>
@@ -5852,8 +5920,20 @@
       <c r="F157" s="4" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="158" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="G157" t="s">
+        <v>565</v>
+      </c>
+      <c r="H157" t="s">
+        <v>566</v>
+      </c>
+      <c r="I157" t="s">
+        <v>567</v>
+      </c>
+      <c r="J157" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" ht="12.75">
       <c r="A158" s="12">
         <v>157</v>
       </c>
@@ -5873,7 +5953,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:10" ht="12.75">
       <c r="A159" s="12">
         <v>158</v>
       </c>
@@ -5893,7 +5973,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:10" ht="12.75">
       <c r="A160" s="12">
         <v>159</v>
       </c>
@@ -5919,7 +5999,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:9" ht="12.75">
       <c r="A161" s="12">
         <v>160</v>
       </c>
@@ -5939,7 +6019,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:9" ht="12.75">
       <c r="A162" s="12">
         <v>161</v>
       </c>
@@ -5959,7 +6039,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:9" ht="12.75">
       <c r="A163" s="12">
         <v>162</v>
       </c>
@@ -5979,7 +6059,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:9" ht="12.75">
       <c r="A164" s="12">
         <v>163</v>
       </c>
@@ -5999,7 +6079,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:9" ht="12.75">
       <c r="A165" s="12">
         <v>164</v>
       </c>
@@ -6019,7 +6099,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:9" ht="12.75">
       <c r="A166" s="12">
         <v>165</v>
       </c>
@@ -6039,7 +6119,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:9" ht="12.75">
       <c r="A167" s="12">
         <v>166</v>
       </c>
@@ -6059,7 +6139,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:9" ht="12.75">
       <c r="A168" s="12">
         <v>167</v>
       </c>
@@ -6079,7 +6159,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:9" ht="12.75">
       <c r="A169" s="12">
         <v>168</v>
       </c>
@@ -6099,7 +6179,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:9" ht="12.75">
       <c r="A170" s="12">
         <v>169</v>
       </c>
@@ -6119,7 +6199,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:9" ht="12.75">
       <c r="A171" s="12">
         <v>170</v>
       </c>
@@ -6139,7 +6219,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:9" ht="12.75">
       <c r="A172" s="12">
         <v>171</v>
       </c>
@@ -6159,7 +6239,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:9" ht="12.75">
       <c r="A173" s="12">
         <v>172</v>
       </c>
@@ -6179,13 +6259,13 @@
         <v>424</v>
       </c>
       <c r="H173" t="s">
+        <v>554</v>
+      </c>
+      <c r="I173" t="s">
         <v>555</v>
       </c>
-      <c r="I173" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="174" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    </row>
+    <row r="174" spans="1:9" ht="12.75">
       <c r="A174" s="12">
         <v>173</v>
       </c>
@@ -6205,7 +6285,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:9" ht="12.75">
       <c r="A175" s="12">
         <v>174</v>
       </c>
@@ -6225,7 +6305,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:9" ht="12.75">
       <c r="A176" s="12">
         <v>175</v>
       </c>
@@ -6245,7 +6325,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="177" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:6" ht="12.75">
       <c r="A177" s="12">
         <v>176</v>
       </c>
@@ -6265,7 +6345,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="178" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:6" ht="12.75">
       <c r="A178" s="12">
         <v>177</v>
       </c>
@@ -6285,7 +6365,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="179" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:6" ht="12.75">
       <c r="A179" s="12">
         <v>178</v>
       </c>
@@ -6305,7 +6385,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="180" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:6" ht="12.75">
       <c r="A180" s="12">
         <v>179</v>
       </c>
@@ -6325,7 +6405,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="181" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:6" ht="12.75">
       <c r="A181" s="12">
         <v>180</v>
       </c>
@@ -6345,7 +6425,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="182" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:6" ht="12.75">
       <c r="A182" s="12">
         <v>181</v>
       </c>
@@ -6365,7 +6445,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="183" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:6" ht="12.75">
       <c r="A183" s="12">
         <v>182</v>
       </c>
@@ -6385,7 +6465,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:6" ht="12.75">
       <c r="A184" s="12">
         <v>183</v>
       </c>
@@ -6405,7 +6485,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="185" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:6" ht="12.75">
       <c r="A185" s="12">
         <v>184</v>
       </c>
@@ -6425,7 +6505,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="186" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:6" ht="12.75">
       <c r="A186" s="12">
         <v>185</v>
       </c>
@@ -6445,7 +6525,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:6" ht="12.75">
       <c r="A187" s="12">
         <v>186</v>
       </c>
@@ -6465,7 +6545,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:6" ht="12.75">
       <c r="A188" s="12">
         <v>187</v>
       </c>
@@ -6485,7 +6565,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:6" ht="12.75">
       <c r="A189" s="12">
         <v>188</v>
       </c>
@@ -6505,7 +6585,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:6" ht="12.75">
       <c r="A190" s="12">
         <v>189</v>
       </c>
@@ -6525,7 +6605,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="191" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:6" ht="12.75">
       <c r="A191" s="12">
         <v>190</v>
       </c>
@@ -6545,7 +6625,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:6" ht="12.75">
       <c r="A192" s="12">
         <v>191</v>
       </c>
@@ -6565,7 +6645,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="193" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:11" ht="12.75">
       <c r="A193" s="12">
         <v>192</v>
       </c>
@@ -6591,7 +6671,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="194" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:11" ht="12.75">
       <c r="A194" s="12">
         <v>193</v>
       </c>
@@ -6617,7 +6697,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="195" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:11" ht="12.75">
       <c r="A195" s="12">
         <v>194</v>
       </c>
@@ -6643,7 +6723,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="196" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:11" ht="12.75">
       <c r="A196" s="12">
         <v>195</v>
       </c>
@@ -6663,7 +6743,7 @@
         <v>486</v>
       </c>
       <c r="G196" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="H196" t="s">
         <v>526</v>
@@ -6678,7 +6758,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="197" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:11" ht="12.75">
       <c r="A197" s="12">
         <v>196</v>
       </c>
@@ -6707,7 +6787,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="198" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:11" ht="12.75">
       <c r="A198" s="12">
         <v>197</v>
       </c>
@@ -6727,7 +6807,7 @@
         <v>486</v>
       </c>
       <c r="G198" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="H198" t="s">
         <v>552</v>
@@ -6736,10 +6816,10 @@
         <v>553</v>
       </c>
       <c r="J198" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="199" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="199" spans="1:11" ht="12.75">
       <c r="A199" s="14">
         <v>1001</v>
       </c>
@@ -6757,7 +6837,7 @@
       </c>
       <c r="F199" s="8"/>
     </row>
-    <row r="200" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:11" ht="12.75">
       <c r="A200" s="14">
         <v>1002</v>
       </c>
@@ -6775,7 +6855,7 @@
       </c>
       <c r="F200" s="8"/>
     </row>
-    <row r="201" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:11" ht="12.75">
       <c r="A201" s="14">
         <v>1003</v>
       </c>
@@ -6791,7 +6871,7 @@
       <c r="E201" s="8"/>
       <c r="F201" s="8"/>
     </row>
-    <row r="202" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:11" ht="12.75">
       <c r="A202" s="14">
         <v>1004</v>
       </c>
@@ -6811,7 +6891,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="203" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:11" ht="12.75">
       <c r="A203" s="14">
         <v>1005</v>
       </c>
@@ -6831,7 +6911,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="204" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:11" ht="12.75">
       <c r="A204" s="15">
         <v>2001</v>
       </c>
@@ -6854,7 +6934,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="205" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:11" ht="12.75">
       <c r="A205" s="15">
         <v>2002</v>
       </c>
@@ -6877,7 +6957,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="206" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:11" ht="12.75">
       <c r="A206" s="15">
         <v>2003</v>
       </c>
@@ -6900,7 +6980,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="207" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:11" ht="12.75">
       <c r="A207" s="15">
         <v>2004</v>
       </c>
@@ -6920,7 +7000,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="208" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:11" ht="13.5" thickBot="1">
       <c r="A208" s="15">
         <v>2005</v>
       </c>
@@ -6940,7 +7020,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="209" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
       <c r="A209" s="16">
         <v>198</v>
       </c>
@@ -6969,7 +7049,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="210" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
       <c r="A210" s="16">
         <v>199</v>
       </c>
@@ -6995,7 +7075,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="211" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
       <c r="A211" s="16">
         <v>200</v>
       </c>
@@ -7027,7 +7107,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="212" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:10" ht="13.5" thickBot="1">
       <c r="A212" s="31">
         <v>201</v>
       </c>
@@ -7059,7 +7139,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="213" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
       <c r="A213" s="33">
         <v>202</v>
       </c>
@@ -7088,7 +7168,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="214" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:10" ht="15.75" customHeight="1">
       <c r="A214" s="30">
         <v>203</v>
       </c>
@@ -7101,12 +7181,14 @@
       <c r="D214" s="27" t="s">
         <v>320</v>
       </c>
-      <c r="E214" s="28"/>
+      <c r="E214" s="28" t="s">
+        <v>564</v>
+      </c>
       <c r="F214" s="27" t="s">
         <v>517</v>
       </c>
       <c r="G214" s="29" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="H214" s="29" t="s">
         <v>522</v>
@@ -7118,41 +7200,99 @@
         <v>524</v>
       </c>
     </row>
-    <row r="215" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:10" ht="15.75" customHeight="1">
       <c r="A215" s="16">
         <v>204</v>
       </c>
       <c r="B215" t="s">
+        <v>556</v>
+      </c>
+      <c r="C215" t="s">
         <v>557</v>
-      </c>
-      <c r="C215" t="s">
-        <v>558</v>
       </c>
       <c r="D215" s="34" t="s">
         <v>245</v>
       </c>
       <c r="E215" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="F215" t="s">
         <v>438</v>
       </c>
       <c r="G215" t="s">
-        <v>561</v>
+        <v>560</v>
+      </c>
+      <c r="H215" t="s">
+        <v>582</v>
+      </c>
+      <c r="I215" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="216" spans="1:10" ht="15.75" customHeight="1">
+      <c r="A216" s="16">
+        <v>205</v>
+      </c>
+      <c r="C216" t="s">
+        <v>571</v>
+      </c>
+      <c r="D216" t="s">
+        <v>569</v>
+      </c>
+      <c r="E216" s="34" t="s">
+        <v>448</v>
+      </c>
+      <c r="F216" t="s">
+        <v>570</v>
+      </c>
+      <c r="H216" t="s">
+        <v>579</v>
+      </c>
+      <c r="I216" t="s">
+        <v>580</v>
+      </c>
+      <c r="J216" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="217" spans="1:10" ht="15.75" customHeight="1">
+      <c r="A217" s="16">
+        <v>206</v>
+      </c>
+      <c r="C217" t="s">
+        <v>572</v>
+      </c>
+      <c r="D217" t="s">
+        <v>569</v>
+      </c>
+      <c r="E217" s="34" t="s">
+        <v>448</v>
+      </c>
+      <c r="F217" t="s">
+        <v>570</v>
+      </c>
+      <c r="H217" t="s">
+        <v>576</v>
+      </c>
+      <c r="I217" t="s">
+        <v>577</v>
+      </c>
+      <c r="J217" t="s">
+        <v>578</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A211 A214" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A211 A214">
       <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E186" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E197" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="E198" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="E209" r:id="rId4" display="http://atotxa.org/" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="E210" r:id="rId5" display="http://atotxa.org/" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E186" r:id="rId1"/>
+    <hyperlink ref="E197" r:id="rId2"/>
+    <hyperlink ref="E198" r:id="rId3"/>
+    <hyperlink ref="E209" r:id="rId4" display="http://atotxa.org/"/>
+    <hyperlink ref="E210" r:id="rId5" display="http://atotxa.org/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>

</xml_diff>

<commit_message>
Romanian club names added to database
</commit_message>
<xml_diff>
--- a/Bufanda Bilduma.xlsx
+++ b/Bufanda Bilduma.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="586">
   <si>
     <t>ZENBAKIA</t>
   </si>
@@ -1840,6 +1840,12 @@
   </si>
   <si>
     <t>atlanta.jpg</t>
+  </si>
+  <si>
+    <t>CFR Cluj</t>
+  </si>
+  <si>
+    <t>FC Hermannstadt</t>
   </si>
 </sst>
 </file>
@@ -7233,6 +7239,9 @@
       <c r="A216" s="16">
         <v>205</v>
       </c>
+      <c r="B216" t="s">
+        <v>584</v>
+      </c>
       <c r="C216" t="s">
         <v>571</v>
       </c>
@@ -7258,6 +7267,9 @@
     <row r="217" spans="1:10" ht="15.75" customHeight="1">
       <c r="A217" s="16">
         <v>206</v>
+      </c>
+      <c r="B217" t="s">
+        <v>585</v>
       </c>
       <c r="C217" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Irudi gehiago. Klik egin eta bilaketara.
</commit_message>
<xml_diff>
--- a/Bufanda Bilduma.xlsx
+++ b/Bufanda Bilduma.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="599">
   <si>
     <t>ZENBAKIA</t>
   </si>
@@ -1846,6 +1846,45 @@
   </si>
   <si>
     <t>FC Hermannstadt</t>
+  </si>
+  <si>
+    <t>Liverpool FC</t>
+  </si>
+  <si>
+    <t>Dortmund</t>
+  </si>
+  <si>
+    <t>Asier Huegun</t>
+  </si>
+  <si>
+    <t>2025 Uztaila</t>
+  </si>
+  <si>
+    <t>2001eko Uefa koparen finalean aldatutako bufanda. Alavesen kamixeta itsusia omen zen eta Asierrek nahiago izan zuen bufanda honekin itzuli Dortmundeko finaletik</t>
+  </si>
+  <si>
+    <t>liverpool_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>liverpool.jpg</t>
+  </si>
+  <si>
+    <t>KuadriJAHrekin Madrila egindako bidaian ekarritako bufanda</t>
+  </si>
+  <si>
+    <t>rayo_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>rayo.jpg</t>
+  </si>
+  <si>
+    <t>Gurasoek Moskura egindako bidaian lortutako 4 bufandetako bat</t>
+  </si>
+  <si>
+    <t>spartak_moskow_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>spartak_moskow.jpg</t>
   </si>
 </sst>
 </file>
@@ -2819,7 +2858,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K217"/>
+  <dimension ref="A1:K218"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="16" customWidth="1"/>
@@ -5335,7 +5374,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="12.75">
+    <row r="129" spans="1:9" ht="12.75">
       <c r="A129" s="12">
         <v>128</v>
       </c>
@@ -5355,7 +5394,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="12.75">
+    <row r="130" spans="1:9" ht="12.75">
       <c r="A130" s="12">
         <v>129</v>
       </c>
@@ -5375,7 +5414,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="12.75">
+    <row r="131" spans="1:9" ht="12.75">
       <c r="A131" s="12">
         <v>130</v>
       </c>
@@ -5395,7 +5434,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="12.75">
+    <row r="132" spans="1:9" ht="12.75">
       <c r="A132" s="12">
         <v>131</v>
       </c>
@@ -5415,7 +5454,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="12.75">
+    <row r="133" spans="1:9" ht="12.75">
       <c r="A133" s="12">
         <v>132</v>
       </c>
@@ -5435,7 +5474,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="12.75">
+    <row r="134" spans="1:9" ht="12.75">
       <c r="A134" s="12">
         <v>133</v>
       </c>
@@ -5458,7 +5497,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="12.75">
+    <row r="135" spans="1:9" ht="12.75">
       <c r="A135" s="12">
         <v>134</v>
       </c>
@@ -5478,7 +5517,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="12.75">
+    <row r="136" spans="1:9" ht="12.75">
       <c r="A136" s="12">
         <v>135</v>
       </c>
@@ -5498,7 +5537,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="12.75">
+    <row r="137" spans="1:9" ht="12.75">
       <c r="A137" s="12">
         <v>136</v>
       </c>
@@ -5518,7 +5557,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="12.75">
+    <row r="138" spans="1:9" ht="12.75">
       <c r="A138" s="12">
         <v>137</v>
       </c>
@@ -5538,7 +5577,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="12.75">
+    <row r="139" spans="1:9" ht="12.75">
       <c r="A139" s="12">
         <v>138</v>
       </c>
@@ -5557,8 +5596,11 @@
       <c r="F139" s="4" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="140" spans="1:7" ht="12.75">
+      <c r="G139" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" ht="12.75">
       <c r="A140" s="12">
         <v>139</v>
       </c>
@@ -5577,8 +5619,11 @@
       <c r="F140" s="3" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="141" spans="1:7" ht="12.75">
+      <c r="G140" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" ht="12.75">
       <c r="A141" s="12">
         <v>140</v>
       </c>
@@ -5597,8 +5642,11 @@
       <c r="F141" s="4" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="142" spans="1:7" ht="12.75">
+      <c r="G141" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" ht="12.75">
       <c r="A142" s="12">
         <v>141</v>
       </c>
@@ -5617,8 +5665,17 @@
       <c r="F142" s="3" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="143" spans="1:7" ht="12.75">
+      <c r="G142" t="s">
+        <v>596</v>
+      </c>
+      <c r="H142" t="s">
+        <v>597</v>
+      </c>
+      <c r="I142" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" ht="12.75">
       <c r="A143" s="12">
         <v>142</v>
       </c>
@@ -5638,7 +5695,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="12.75">
+    <row r="144" spans="1:9" ht="12.75">
       <c r="A144" s="12">
         <v>143</v>
       </c>
@@ -5677,6 +5734,15 @@
       <c r="F145" s="4" t="s">
         <v>347</v>
       </c>
+      <c r="G145" t="s">
+        <v>593</v>
+      </c>
+      <c r="H145" t="s">
+        <v>594</v>
+      </c>
+      <c r="I145" t="s">
+        <v>595</v>
+      </c>
     </row>
     <row r="146" spans="1:10" ht="12.75">
       <c r="A146" s="12">
@@ -7291,6 +7357,35 @@
       </c>
       <c r="J217" t="s">
         <v>578</v>
+      </c>
+    </row>
+    <row r="218" spans="1:10" ht="15.75" customHeight="1">
+      <c r="A218" s="16">
+        <v>207</v>
+      </c>
+      <c r="B218" t="s">
+        <v>586</v>
+      </c>
+      <c r="C218" t="s">
+        <v>587</v>
+      </c>
+      <c r="D218" t="s">
+        <v>90</v>
+      </c>
+      <c r="E218" t="s">
+        <v>588</v>
+      </c>
+      <c r="F218" t="s">
+        <v>589</v>
+      </c>
+      <c r="G218" t="s">
+        <v>590</v>
+      </c>
+      <c r="H218" t="s">
+        <v>591</v>
+      </c>
+      <c r="I218" t="s">
+        <v>592</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
racing de santander added
</commit_message>
<xml_diff>
--- a/Bufanda Bilduma.xlsx
+++ b/Bufanda Bilduma.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Kodea\Beste\bufandaweb2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andmu\Documents\Andoni\kodea\bufandaweb\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B6BF7E-295A-47CB-86F0-67E6CDB385C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="657">
   <si>
     <t>ZENBAKIA</t>
   </si>
@@ -2040,12 +2041,33 @@
   <si>
     <t>bayern.jpg</t>
   </si>
+  <si>
+    <t>Atotxa.org eta Ciclista Footbal Clubeko bi frikiek ateratako bufanda</t>
+  </si>
+  <si>
+    <t>2025 Azaroa</t>
+  </si>
+  <si>
+    <t>Estitxu eta Asier Santanderrera joan ziren Anari eta Uxeu euskal selekzioarekin ikustera</t>
+  </si>
+  <si>
+    <t>Racing de Santander</t>
+  </si>
+  <si>
+    <t>Santander</t>
+  </si>
+  <si>
+    <t>racing_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>racing.jpg</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2692,7 +2714,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle name="Sheet1-style" pivot="0" count="3">
+    <tableStyle name="Sheet1-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="headerRow" dxfId="3"/>
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="secondRowStripe" dxfId="1"/>
@@ -2710,19 +2732,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:K213">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K213">
   <tableColumns count="11">
-    <tableColumn id="1" name="ZENBAKIA" dataDxfId="0"/>
-    <tableColumn id="2" name="TALDEA"/>
-    <tableColumn id="3" name="NONDIK"/>
-    <tableColumn id="4" name="LIGA"/>
-    <tableColumn id="5" name="NORK"/>
-    <tableColumn id="6" name="NOIZ"/>
-    <tableColumn id="7" name="BESTE"/>
-    <tableColumn id="8" name="main_image"/>
-    <tableColumn id="9" name="image_1"/>
-    <tableColumn id="10" name="image_2"/>
-    <tableColumn id="11" name="image_3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ZENBAKIA" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="TALDEA"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="NONDIK"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="LIGA"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="NORK"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="NOIZ"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="BESTE"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="main_image"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="image_1"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="image_2"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="image_3"/>
   </tableColumns>
   <tableStyleInfo name="Sheet1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3044,12 +3066,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K220"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:K221"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="16" customWidth="1"/>
     <col min="2" max="2" width="40.28515625" bestFit="1" customWidth="1"/>
@@ -3064,7 +3086,7 @@
     <col min="11" max="11" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" customHeight="1">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -3099,7 +3121,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -3134,7 +3156,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12">
         <v>2</v>
       </c>
@@ -3154,7 +3176,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12">
         <v>3</v>
       </c>
@@ -3174,7 +3196,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -3194,7 +3216,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1">
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12">
         <v>5</v>
       </c>
@@ -3214,7 +3236,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -3231,7 +3253,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1">
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12">
         <v>7</v>
       </c>
@@ -3254,7 +3276,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1">
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12">
         <v>8</v>
       </c>
@@ -3274,7 +3296,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1">
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="12">
         <v>9</v>
       </c>
@@ -3294,7 +3316,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1">
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="12">
         <v>10</v>
       </c>
@@ -3314,7 +3336,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1">
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12">
         <v>11</v>
       </c>
@@ -3331,7 +3353,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1">
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12">
         <v>12</v>
       </c>
@@ -3348,7 +3370,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1">
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12">
         <v>13</v>
       </c>
@@ -3368,7 +3390,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1">
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="12">
         <v>14</v>
       </c>
@@ -3388,7 +3410,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1">
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12">
         <v>15</v>
       </c>
@@ -3408,7 +3430,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="12">
         <v>16</v>
       </c>
@@ -3422,7 +3444,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="12">
         <v>17</v>
       </c>
@@ -3442,7 +3464,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15.75" customHeight="1">
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12">
         <v>18</v>
       </c>
@@ -3459,7 +3481,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="12">
         <v>19</v>
       </c>
@@ -3476,7 +3498,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="12">
         <v>20</v>
       </c>
@@ -3496,7 +3518,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12">
         <v>21</v>
       </c>
@@ -3516,7 +3538,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="12">
         <v>22</v>
       </c>
@@ -3536,7 +3558,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="12">
         <v>23</v>
       </c>
@@ -3553,7 +3575,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="12">
         <v>24</v>
       </c>
@@ -3570,7 +3592,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="15.75" customHeight="1">
+    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="12">
         <v>25</v>
       </c>
@@ -3590,7 +3612,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12">
         <v>26</v>
       </c>
@@ -3610,7 +3632,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="12">
         <v>27</v>
       </c>
@@ -3627,7 +3649,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="12">
         <v>28</v>
       </c>
@@ -3644,7 +3666,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="12">
         <v>29</v>
       </c>
@@ -3661,7 +3683,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15.75" customHeight="1">
+    <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="12">
         <v>30</v>
       </c>
@@ -3678,7 +3700,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15.75" customHeight="1">
+    <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="12">
         <v>31</v>
       </c>
@@ -3695,7 +3717,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="15.75" customHeight="1">
+    <row r="33" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="12">
         <v>32</v>
       </c>
@@ -3715,7 +3737,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75" customHeight="1">
+    <row r="34" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="12">
         <v>33</v>
       </c>
@@ -3735,7 +3757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15.75" customHeight="1">
+    <row r="35" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="12">
         <v>34</v>
       </c>
@@ -3752,7 +3774,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="15.75" customHeight="1">
+    <row r="36" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="12">
         <v>35</v>
       </c>
@@ -3772,7 +3794,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="15.75" customHeight="1">
+    <row r="37" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="12">
         <v>36</v>
       </c>
@@ -3792,7 +3814,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="12.75">
+    <row r="38" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="12">
         <v>37</v>
       </c>
@@ -3821,7 +3843,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="12.75">
+    <row r="39" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="12">
         <v>38</v>
       </c>
@@ -3838,7 +3860,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="12.75">
+    <row r="40" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="12">
         <v>39</v>
       </c>
@@ -3858,7 +3880,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="12.75">
+    <row r="41" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="12">
         <v>40</v>
       </c>
@@ -3878,7 +3900,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="12.75">
+    <row r="42" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="12">
         <v>41</v>
       </c>
@@ -3895,7 +3917,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="12.75">
+    <row r="43" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="12">
         <v>42</v>
       </c>
@@ -3915,7 +3937,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="12.75">
+    <row r="44" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="12">
         <v>43</v>
       </c>
@@ -3935,7 +3957,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="12.75">
+    <row r="45" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="12">
         <v>44</v>
       </c>
@@ -3955,7 +3977,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="12.75">
+    <row r="46" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A46" s="12">
         <v>45</v>
       </c>
@@ -3972,7 +3994,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="12.75">
+    <row r="47" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A47" s="12">
         <v>46</v>
       </c>
@@ -3989,7 +4011,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="12.75">
+    <row r="48" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A48" s="12">
         <v>47</v>
       </c>
@@ -4009,7 +4031,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="12.75">
+    <row r="49" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A49" s="12">
         <v>48</v>
       </c>
@@ -4026,7 +4048,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="12.75">
+    <row r="50" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A50" s="12">
         <v>49</v>
       </c>
@@ -4046,7 +4068,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="12.75">
+    <row r="51" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A51" s="12">
         <v>50</v>
       </c>
@@ -4066,7 +4088,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="12.75">
+    <row r="52" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A52" s="12">
         <v>51</v>
       </c>
@@ -4083,7 +4105,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="12.75">
+    <row r="53" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A53" s="12">
         <v>52</v>
       </c>
@@ -4103,7 +4125,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="12.75">
+    <row r="54" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A54" s="12">
         <v>53</v>
       </c>
@@ -4120,7 +4142,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="12.75">
+    <row r="55" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A55" s="12">
         <v>54</v>
       </c>
@@ -4140,7 +4162,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="12.75">
+    <row r="56" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A56" s="12">
         <v>55</v>
       </c>
@@ -4160,7 +4182,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="12.75">
+    <row r="57" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A57" s="12">
         <v>56</v>
       </c>
@@ -4180,7 +4202,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="12.75">
+    <row r="58" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A58" s="12">
         <v>57</v>
       </c>
@@ -4200,7 +4222,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="12.75">
+    <row r="59" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A59" s="12">
         <v>58</v>
       </c>
@@ -4217,7 +4239,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="12.75">
+    <row r="60" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A60" s="12">
         <v>59</v>
       </c>
@@ -4234,7 +4256,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="12.75">
+    <row r="61" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A61" s="12">
         <v>60</v>
       </c>
@@ -4254,7 +4276,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="12.75">
+    <row r="62" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A62" s="12">
         <v>61</v>
       </c>
@@ -4274,7 +4296,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="12.75">
+    <row r="63" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A63" s="12">
         <v>62</v>
       </c>
@@ -4294,7 +4316,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="12.75">
+    <row r="64" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A64" s="12">
         <v>63</v>
       </c>
@@ -4314,7 +4336,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="12.75">
+    <row r="65" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A65" s="12">
         <v>64</v>
       </c>
@@ -4346,7 +4368,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="12.75">
+    <row r="66" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A66" s="12">
         <v>65</v>
       </c>
@@ -4366,7 +4388,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="12.75">
+    <row r="67" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A67" s="12">
         <v>66</v>
       </c>
@@ -4386,7 +4408,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="12.75">
+    <row r="68" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A68" s="12">
         <v>67</v>
       </c>
@@ -4406,7 +4428,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="12.75">
+    <row r="69" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A69" s="12">
         <v>68</v>
       </c>
@@ -4426,7 +4448,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="12.75">
+    <row r="70" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A70" s="12">
         <v>69</v>
       </c>
@@ -4446,7 +4468,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="12.75">
+    <row r="71" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A71" s="12">
         <v>70</v>
       </c>
@@ -4466,7 +4488,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="12.75">
+    <row r="72" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A72" s="12">
         <v>71</v>
       </c>
@@ -4486,7 +4508,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="12.75">
+    <row r="73" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A73" s="12">
         <v>72</v>
       </c>
@@ -4506,7 +4528,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="12.75">
+    <row r="74" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A74" s="12">
         <v>73</v>
       </c>
@@ -4526,7 +4548,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="12.75">
+    <row r="75" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A75" s="12">
         <v>74</v>
       </c>
@@ -4546,7 +4568,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="12.75">
+    <row r="76" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A76" s="12">
         <v>75</v>
       </c>
@@ -4566,7 +4588,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="12.75">
+    <row r="77" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A77" s="12">
         <v>76</v>
       </c>
@@ -4586,7 +4608,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="12.75">
+    <row r="78" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A78" s="12">
         <v>77</v>
       </c>
@@ -4606,7 +4628,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="12.75">
+    <row r="79" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A79" s="12">
         <v>78</v>
       </c>
@@ -4626,7 +4648,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="12.75">
+    <row r="80" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A80" s="12">
         <v>79</v>
       </c>
@@ -4646,7 +4668,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="12.75">
+    <row r="81" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A81" s="12">
         <v>80</v>
       </c>
@@ -4666,7 +4688,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="12.75">
+    <row r="82" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A82" s="12">
         <v>81</v>
       </c>
@@ -4686,7 +4708,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="12.75">
+    <row r="83" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A83" s="12">
         <v>82</v>
       </c>
@@ -4706,7 +4728,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="12.75">
+    <row r="84" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A84" s="12">
         <v>83</v>
       </c>
@@ -4726,7 +4748,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="12.75">
+    <row r="85" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A85" s="12">
         <v>84</v>
       </c>
@@ -4746,7 +4768,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="12.75">
+    <row r="86" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A86" s="12">
         <v>85</v>
       </c>
@@ -4766,7 +4788,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="12.75">
+    <row r="87" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A87" s="12">
         <v>86</v>
       </c>
@@ -4786,7 +4808,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="12.75">
+    <row r="88" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A88" s="12">
         <v>87</v>
       </c>
@@ -4806,7 +4828,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="12.75">
+    <row r="89" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A89" s="12">
         <v>88</v>
       </c>
@@ -4829,7 +4851,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="12.75">
+    <row r="90" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A90" s="12">
         <v>89</v>
       </c>
@@ -4852,7 +4874,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="12.75">
+    <row r="91" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A91" s="12">
         <v>90</v>
       </c>
@@ -4875,7 +4897,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="12.75">
+    <row r="92" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A92" s="12">
         <v>91</v>
       </c>
@@ -4898,7 +4920,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="12.75">
+    <row r="93" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A93" s="12">
         <v>92</v>
       </c>
@@ -4921,7 +4943,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="12.75">
+    <row r="94" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A94" s="12">
         <v>93</v>
       </c>
@@ -4944,7 +4966,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="12.75">
+    <row r="95" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A95" s="12">
         <v>94</v>
       </c>
@@ -4973,7 +4995,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="12.75">
+    <row r="96" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A96" s="12">
         <v>95</v>
       </c>
@@ -5002,7 +5024,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="12.75">
+    <row r="97" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A97" s="12">
         <v>96</v>
       </c>
@@ -5025,7 +5047,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="12.75">
+    <row r="98" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A98" s="12">
         <v>97</v>
       </c>
@@ -5048,7 +5070,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="12.75">
+    <row r="99" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A99" s="12">
         <v>98</v>
       </c>
@@ -5071,7 +5093,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="12.75">
+    <row r="100" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A100" s="12">
         <v>99</v>
       </c>
@@ -5094,7 +5116,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="12.75">
+    <row r="101" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A101" s="12">
         <v>100</v>
       </c>
@@ -5114,7 +5136,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="12.75">
+    <row r="102" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A102" s="12">
         <v>101</v>
       </c>
@@ -5134,7 +5156,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="12.75">
+    <row r="103" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A103" s="12">
         <v>102</v>
       </c>
@@ -5154,7 +5176,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="12.75">
+    <row r="104" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A104" s="12">
         <v>103</v>
       </c>
@@ -5174,7 +5196,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="12.75">
+    <row r="105" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A105" s="12">
         <v>104</v>
       </c>
@@ -5194,7 +5216,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="12.75">
+    <row r="106" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A106" s="12">
         <v>105</v>
       </c>
@@ -5214,7 +5236,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="12.75">
+    <row r="107" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A107" s="12">
         <v>106</v>
       </c>
@@ -5234,7 +5256,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="12.75">
+    <row r="108" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A108" s="12">
         <v>107</v>
       </c>
@@ -5254,7 +5276,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="12.75">
+    <row r="109" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A109" s="12">
         <v>108</v>
       </c>
@@ -5274,7 +5296,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="12.75">
+    <row r="110" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A110" s="12">
         <v>109</v>
       </c>
@@ -5294,7 +5316,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="12.75">
+    <row r="111" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A111" s="12">
         <v>110</v>
       </c>
@@ -5314,7 +5336,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="12.75">
+    <row r="112" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A112" s="12">
         <v>111</v>
       </c>
@@ -5334,7 +5356,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="12.75">
+    <row r="113" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A113" s="12">
         <v>112</v>
       </c>
@@ -5354,7 +5376,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="12.75">
+    <row r="114" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A114" s="12">
         <v>113</v>
       </c>
@@ -5374,7 +5396,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="12.75">
+    <row r="115" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A115" s="12">
         <v>114</v>
       </c>
@@ -5394,7 +5416,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="12.75">
+    <row r="116" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A116" s="12">
         <v>115</v>
       </c>
@@ -5414,7 +5436,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="12.75">
+    <row r="117" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A117" s="12">
         <v>116</v>
       </c>
@@ -5434,7 +5456,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="12.75">
+    <row r="118" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A118" s="12">
         <v>117</v>
       </c>
@@ -5454,7 +5476,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="12.75">
+    <row r="119" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A119" s="12">
         <v>118</v>
       </c>
@@ -5483,7 +5505,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="12.75">
+    <row r="120" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A120" s="12">
         <v>119</v>
       </c>
@@ -5503,7 +5525,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="12.75">
+    <row r="121" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A121" s="12">
         <v>120</v>
       </c>
@@ -5523,7 +5545,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="12.75">
+    <row r="122" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A122" s="12">
         <v>121</v>
       </c>
@@ -5543,7 +5565,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="12.75">
+    <row r="123" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A123" s="12">
         <v>122</v>
       </c>
@@ -5563,7 +5585,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="12.75">
+    <row r="124" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A124" s="12">
         <v>123</v>
       </c>
@@ -5583,7 +5605,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="12.75">
+    <row r="125" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A125" s="12">
         <v>124</v>
       </c>
@@ -5603,7 +5625,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="12.75">
+    <row r="126" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A126" s="12">
         <v>125</v>
       </c>
@@ -5623,7 +5645,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="12.75">
+    <row r="127" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A127" s="12">
         <v>126</v>
       </c>
@@ -5643,7 +5665,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="12.75">
+    <row r="128" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A128" s="12">
         <v>127</v>
       </c>
@@ -5663,7 +5685,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="129" spans="1:11" ht="12.75">
+    <row r="129" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A129" s="12">
         <v>128</v>
       </c>
@@ -5683,7 +5705,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="130" spans="1:11" ht="12.75">
+    <row r="130" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A130" s="12">
         <v>129</v>
       </c>
@@ -5703,7 +5725,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="131" spans="1:11" ht="12.75">
+    <row r="131" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A131" s="12">
         <v>130</v>
       </c>
@@ -5723,7 +5745,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="132" spans="1:11" ht="12.75">
+    <row r="132" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A132" s="12">
         <v>131</v>
       </c>
@@ -5743,7 +5765,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="133" spans="1:11" ht="12.75">
+    <row r="133" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A133" s="12">
         <v>132</v>
       </c>
@@ -5763,7 +5785,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="134" spans="1:11" ht="12.75">
+    <row r="134" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A134" s="12">
         <v>133</v>
       </c>
@@ -5786,7 +5808,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="135" spans="1:11" ht="12.75">
+    <row r="135" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A135" s="12">
         <v>134</v>
       </c>
@@ -5806,7 +5828,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="136" spans="1:11" ht="12.75">
+    <row r="136" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A136" s="12">
         <v>135</v>
       </c>
@@ -5826,7 +5848,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="137" spans="1:11" ht="12.75">
+    <row r="137" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A137" s="12">
         <v>136</v>
       </c>
@@ -5846,7 +5868,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="138" spans="1:11" ht="12.75">
+    <row r="138" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A138" s="12">
         <v>137</v>
       </c>
@@ -5866,7 +5888,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="139" spans="1:11" ht="12.75">
+    <row r="139" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A139" s="12">
         <v>138</v>
       </c>
@@ -5889,7 +5911,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="140" spans="1:11" ht="12.75">
+    <row r="140" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A140" s="12">
         <v>139</v>
       </c>
@@ -5918,7 +5940,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="141" spans="1:11" ht="12.75">
+    <row r="141" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A141" s="12">
         <v>140</v>
       </c>
@@ -5953,7 +5975,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="142" spans="1:11" ht="12.75">
+    <row r="142" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A142" s="12">
         <v>141</v>
       </c>
@@ -5982,7 +6004,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="143" spans="1:11" ht="12.75">
+    <row r="143" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A143" s="12">
         <v>142</v>
       </c>
@@ -6002,7 +6024,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="144" spans="1:11" ht="12.75">
+    <row r="144" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A144" s="12">
         <v>143</v>
       </c>
@@ -6022,7 +6044,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="12.75">
+    <row r="145" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A145" s="12">
         <v>144</v>
       </c>
@@ -6051,7 +6073,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="12.75">
+    <row r="146" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A146" s="12">
         <v>145</v>
       </c>
@@ -6071,7 +6093,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="12.75">
+    <row r="147" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A147" s="12">
         <v>146</v>
       </c>
@@ -6091,7 +6113,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="12.75">
+    <row r="148" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A148" s="12">
         <v>147</v>
       </c>
@@ -6111,7 +6133,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="12.75">
+    <row r="149" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A149" s="12">
         <v>148</v>
       </c>
@@ -6131,7 +6153,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="12.75">
+    <row r="150" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A150" s="12">
         <v>149</v>
       </c>
@@ -6151,7 +6173,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="12.75">
+    <row r="151" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A151" s="12">
         <v>150</v>
       </c>
@@ -6171,7 +6193,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="12.75">
+    <row r="152" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A152" s="12">
         <v>151</v>
       </c>
@@ -6191,7 +6213,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="12.75">
+    <row r="153" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A153" s="12">
         <v>152</v>
       </c>
@@ -6223,7 +6245,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="12.75">
+    <row r="154" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A154" s="12">
         <v>153</v>
       </c>
@@ -6243,7 +6265,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="12.75">
+    <row r="155" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A155" s="12">
         <v>154</v>
       </c>
@@ -6263,7 +6285,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="12.75">
+    <row r="156" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A156" s="12">
         <v>155</v>
       </c>
@@ -6292,7 +6314,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="157" spans="1:10" ht="12.75">
+    <row r="157" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A157" s="12">
         <v>156</v>
       </c>
@@ -6324,7 +6346,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="12.75">
+    <row r="158" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A158" s="12">
         <v>157</v>
       </c>
@@ -6344,7 +6366,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="12.75">
+    <row r="159" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A159" s="12">
         <v>158</v>
       </c>
@@ -6364,7 +6386,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="12.75">
+    <row r="160" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A160" s="12">
         <v>159</v>
       </c>
@@ -6390,7 +6412,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="12.75">
+    <row r="161" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A161" s="12">
         <v>160</v>
       </c>
@@ -6410,7 +6432,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="12.75">
+    <row r="162" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A162" s="12">
         <v>161</v>
       </c>
@@ -6430,7 +6452,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="12.75">
+    <row r="163" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A163" s="12">
         <v>162</v>
       </c>
@@ -6450,7 +6472,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="12.75">
+    <row r="164" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A164" s="12">
         <v>163</v>
       </c>
@@ -6470,7 +6492,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="12.75">
+    <row r="165" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A165" s="12">
         <v>164</v>
       </c>
@@ -6490,7 +6512,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="12.75">
+    <row r="166" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A166" s="12">
         <v>165</v>
       </c>
@@ -6510,7 +6532,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="12.75">
+    <row r="167" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A167" s="12">
         <v>166</v>
       </c>
@@ -6530,7 +6552,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="12.75">
+    <row r="168" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A168" s="12">
         <v>167</v>
       </c>
@@ -6550,7 +6572,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="12.75">
+    <row r="169" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A169" s="12">
         <v>168</v>
       </c>
@@ -6570,7 +6592,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="12.75">
+    <row r="170" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A170" s="12">
         <v>169</v>
       </c>
@@ -6590,7 +6612,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="12.75">
+    <row r="171" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A171" s="12">
         <v>170</v>
       </c>
@@ -6610,7 +6632,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="12.75">
+    <row r="172" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A172" s="12">
         <v>171</v>
       </c>
@@ -6630,7 +6652,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="12.75">
+    <row r="173" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A173" s="12">
         <v>172</v>
       </c>
@@ -6656,7 +6678,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="12.75">
+    <row r="174" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A174" s="12">
         <v>173</v>
       </c>
@@ -6676,7 +6698,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="12.75">
+    <row r="175" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A175" s="12">
         <v>174</v>
       </c>
@@ -6696,7 +6718,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="12.75">
+    <row r="176" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A176" s="12">
         <v>175</v>
       </c>
@@ -6716,7 +6738,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="177" spans="1:6" ht="12.75">
+    <row r="177" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A177" s="12">
         <v>176</v>
       </c>
@@ -6736,7 +6758,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="178" spans="1:6" ht="12.75">
+    <row r="178" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A178" s="12">
         <v>177</v>
       </c>
@@ -6756,7 +6778,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="179" spans="1:6" ht="12.75">
+    <row r="179" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A179" s="12">
         <v>178</v>
       </c>
@@ -6776,7 +6798,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="180" spans="1:6" ht="12.75">
+    <row r="180" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A180" s="12">
         <v>179</v>
       </c>
@@ -6796,7 +6818,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="181" spans="1:6" ht="12.75">
+    <row r="181" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A181" s="12">
         <v>180</v>
       </c>
@@ -6816,7 +6838,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="182" spans="1:6" ht="12.75">
+    <row r="182" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A182" s="12">
         <v>181</v>
       </c>
@@ -6836,7 +6858,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="183" spans="1:6" ht="12.75">
+    <row r="183" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A183" s="12">
         <v>182</v>
       </c>
@@ -6856,7 +6878,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ht="12.75">
+    <row r="184" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A184" s="12">
         <v>183</v>
       </c>
@@ -6876,7 +6898,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="185" spans="1:6" ht="12.75">
+    <row r="185" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A185" s="12">
         <v>184</v>
       </c>
@@ -6896,7 +6918,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="186" spans="1:6" ht="12.75">
+    <row r="186" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A186" s="12">
         <v>185</v>
       </c>
@@ -6916,7 +6938,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ht="12.75">
+    <row r="187" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A187" s="12">
         <v>186</v>
       </c>
@@ -6936,7 +6958,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ht="12.75">
+    <row r="188" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A188" s="12">
         <v>187</v>
       </c>
@@ -6956,7 +6978,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ht="12.75">
+    <row r="189" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A189" s="12">
         <v>188</v>
       </c>
@@ -6976,7 +6998,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="12.75">
+    <row r="190" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A190" s="12">
         <v>189</v>
       </c>
@@ -6996,7 +7018,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="191" spans="1:6" ht="12.75">
+    <row r="191" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A191" s="12">
         <v>190</v>
       </c>
@@ -7016,7 +7038,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="12.75">
+    <row r="192" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A192" s="12">
         <v>191</v>
       </c>
@@ -7036,7 +7058,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="193" spans="1:11" ht="12.75">
+    <row r="193" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A193" s="12">
         <v>192</v>
       </c>
@@ -7062,7 +7084,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="194" spans="1:11" ht="12.75">
+    <row r="194" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A194" s="12">
         <v>193</v>
       </c>
@@ -7088,7 +7110,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="195" spans="1:11" ht="12.75">
+    <row r="195" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A195" s="12">
         <v>194</v>
       </c>
@@ -7114,7 +7136,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="196" spans="1:11" ht="12.75">
+    <row r="196" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A196" s="12">
         <v>195</v>
       </c>
@@ -7149,7 +7171,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="197" spans="1:11" ht="12.75">
+    <row r="197" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A197" s="12">
         <v>196</v>
       </c>
@@ -7178,7 +7200,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="198" spans="1:11" ht="12.75">
+    <row r="198" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A198" s="12">
         <v>197</v>
       </c>
@@ -7210,7 +7232,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="199" spans="1:11" ht="12.75">
+    <row r="199" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A199" s="14">
         <v>1001</v>
       </c>
@@ -7228,7 +7250,7 @@
       </c>
       <c r="F199" s="8"/>
     </row>
-    <row r="200" spans="1:11" ht="12.75">
+    <row r="200" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A200" s="14">
         <v>1002</v>
       </c>
@@ -7246,7 +7268,7 @@
       </c>
       <c r="F200" s="8"/>
     </row>
-    <row r="201" spans="1:11" ht="12.75">
+    <row r="201" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A201" s="14">
         <v>1003</v>
       </c>
@@ -7262,7 +7284,7 @@
       <c r="E201" s="8"/>
       <c r="F201" s="8"/>
     </row>
-    <row r="202" spans="1:11" ht="12.75">
+    <row r="202" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A202" s="14">
         <v>1004</v>
       </c>
@@ -7282,7 +7304,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="203" spans="1:11" ht="12.75">
+    <row r="203" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A203" s="14">
         <v>1005</v>
       </c>
@@ -7302,7 +7324,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="204" spans="1:11" ht="12.75">
+    <row r="204" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A204" s="15">
         <v>2001</v>
       </c>
@@ -7325,7 +7347,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="205" spans="1:11" ht="12.75">
+    <row r="205" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A205" s="15">
         <v>2002</v>
       </c>
@@ -7348,7 +7370,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="206" spans="1:11" ht="12.75">
+    <row r="206" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A206" s="15">
         <v>2003</v>
       </c>
@@ -7371,7 +7393,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="207" spans="1:11" ht="12.75">
+    <row r="207" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A207" s="15">
         <v>2004</v>
       </c>
@@ -7391,7 +7413,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="208" spans="1:11" ht="13.5" thickBot="1">
+    <row r="208" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A208" s="15">
         <v>2005</v>
       </c>
@@ -7411,7 +7433,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="209" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+    <row r="209" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A209" s="16">
         <v>198</v>
       </c>
@@ -7430,6 +7452,9 @@
       <c r="F209" s="19" t="s">
         <v>513</v>
       </c>
+      <c r="G209" t="s">
+        <v>650</v>
+      </c>
       <c r="H209" t="s">
         <v>537</v>
       </c>
@@ -7440,7 +7465,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="210" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+    <row r="210" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A210" s="16">
         <v>199</v>
       </c>
@@ -7459,6 +7484,9 @@
       <c r="F210" s="22" t="s">
         <v>513</v>
       </c>
+      <c r="G210" t="s">
+        <v>650</v>
+      </c>
       <c r="H210" t="s">
         <v>535</v>
       </c>
@@ -7466,7 +7494,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="211" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+    <row r="211" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A211" s="16">
         <v>200</v>
       </c>
@@ -7498,7 +7526,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="212" spans="1:11" ht="13.5" thickBot="1">
+    <row r="212" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A212" s="31">
         <v>201</v>
       </c>
@@ -7530,7 +7558,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="213" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+    <row r="213" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A213" s="33">
         <v>202</v>
       </c>
@@ -7559,7 +7587,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="214" spans="1:11" ht="15.75" customHeight="1">
+    <row r="214" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="30">
         <v>203</v>
       </c>
@@ -7591,7 +7619,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="215" spans="1:11" ht="15.75" customHeight="1">
+    <row r="215" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="16">
         <v>204</v>
       </c>
@@ -7620,7 +7648,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="216" spans="1:11" ht="15.75" customHeight="1">
+    <row r="216" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="16">
         <v>205</v>
       </c>
@@ -7652,7 +7680,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="217" spans="1:11" ht="15.75" customHeight="1">
+    <row r="217" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="16">
         <v>206</v>
       </c>
@@ -7684,7 +7712,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="218" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+    <row r="218" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A218" s="16">
         <v>207</v>
       </c>
@@ -7713,7 +7741,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="219" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+    <row r="219" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A219" s="16">
         <v>208</v>
       </c>
@@ -7746,7 +7774,7 @@
       </c>
       <c r="K219" s="35"/>
     </row>
-    <row r="220" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+    <row r="220" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A220" s="16">
         <v>209</v>
       </c>
@@ -7781,18 +7809,47 @@
         <v>615</v>
       </c>
     </row>
+    <row r="221" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A221" s="16">
+        <v>210</v>
+      </c>
+      <c r="B221" t="s">
+        <v>653</v>
+      </c>
+      <c r="C221" t="s">
+        <v>654</v>
+      </c>
+      <c r="D221" t="s">
+        <v>51</v>
+      </c>
+      <c r="E221" s="34" t="s">
+        <v>448</v>
+      </c>
+      <c r="F221" t="s">
+        <v>651</v>
+      </c>
+      <c r="G221" t="s">
+        <v>652</v>
+      </c>
+      <c r="H221" t="s">
+        <v>655</v>
+      </c>
+      <c r="I221" t="s">
+        <v>656</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A211 A214">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A211 A214" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E186" r:id="rId1"/>
-    <hyperlink ref="E197" r:id="rId2"/>
-    <hyperlink ref="E198" r:id="rId3"/>
-    <hyperlink ref="E209" r:id="rId4" display="http://atotxa.org/"/>
-    <hyperlink ref="E210" r:id="rId5" display="http://atotxa.org/"/>
+    <hyperlink ref="E186" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E197" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E198" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E209" r:id="rId4" display="http://atotxa.org/" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E210" r:id="rId5" display="http://atotxa.org/" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>

</xml_diff>

<commit_message>
AEK and Japan added.
</commit_message>
<xml_diff>
--- a/Bufanda Bilduma.xlsx
+++ b/Bufanda Bilduma.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andmu\Documents\Andoni\kodea\bufandaweb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966CFBB2-65F2-46D6-854A-04722DFE15ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57397C7-7191-4597-A03F-C878EA40F73E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1243" uniqueCount="677">
   <si>
     <t>ZENBAKIA</t>
   </si>
@@ -2091,6 +2091,36 @@
   </si>
   <si>
     <t>cymru.jpg</t>
+  </si>
+  <si>
+    <t>Jon Haitz Legarreta</t>
+  </si>
+  <si>
+    <t>2025 Urria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jon Haitzek kongresu batera egindako bidaian erositako bufanda. Ziurrenik, bilduma honetan kilometro gehien egin dituen bufanda: Japonia -&gt; Boston -&gt; Gatika -&gt; Donostia. Japoniako beste bufanda bezala, toalla estilokoa da; berezia. </t>
+  </si>
+  <si>
+    <t>japan_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>japan.jpg</t>
+  </si>
+  <si>
+    <t>japan_eskudo_2.jpg</t>
+  </si>
+  <si>
+    <t>AEK Atenas</t>
+  </si>
+  <si>
+    <t>Asierrek lagun batzuk engainatu zituen bufanda hau ekartzeko. Edozer gauza bilduma honetan bere aportazioa handitzeko.</t>
+  </si>
+  <si>
+    <t>aek_eskudo.jpg</t>
+  </si>
+  <si>
+    <t>aek.jpg</t>
   </si>
 </sst>
 </file>
@@ -3100,7 +3130,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K221"/>
+  <dimension ref="A1:K223"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="16" customWidth="1"/>
@@ -7899,6 +7929,67 @@
       </c>
       <c r="I221" t="s">
         <v>655</v>
+      </c>
+    </row>
+    <row r="222" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A222" s="16">
+        <v>211</v>
+      </c>
+      <c r="B222" t="s">
+        <v>429</v>
+      </c>
+      <c r="C222" t="s">
+        <v>428</v>
+      </c>
+      <c r="D222" t="s">
+        <v>121</v>
+      </c>
+      <c r="E222" t="s">
+        <v>667</v>
+      </c>
+      <c r="F222" t="s">
+        <v>668</v>
+      </c>
+      <c r="G222" t="s">
+        <v>669</v>
+      </c>
+      <c r="H222" t="s">
+        <v>670</v>
+      </c>
+      <c r="I222" t="s">
+        <v>671</v>
+      </c>
+      <c r="J222" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="223" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A223" s="16">
+        <v>212</v>
+      </c>
+      <c r="B223" t="s">
+        <v>673</v>
+      </c>
+      <c r="C223" t="s">
+        <v>77</v>
+      </c>
+      <c r="D223" t="s">
+        <v>78</v>
+      </c>
+      <c r="E223" t="s">
+        <v>588</v>
+      </c>
+      <c r="F223" t="s">
+        <v>668</v>
+      </c>
+      <c r="G223" t="s">
+        <v>674</v>
+      </c>
+      <c r="H223" t="s">
+        <v>675</v>
+      </c>
+      <c r="I223" t="s">
+        <v>676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>